<commit_message>
Improve thermo defaults and workbook-driven controls
</commit_message>
<xml_diff>
--- a/sandbox/mini8/input/distillation_column_template_20stage_chemsep_warmer_feed_seed_20260323.xlsx
+++ b/sandbox/mini8/input/distillation_column_template_20stage_chemsep_warmer_feed_seed_20260323.xlsx
@@ -21,7 +21,7 @@
     <numFmt numFmtId="164" formatCode="0.0000"/>
     <numFmt numFmtId="165" formatCode="#,##0.000_);\(#,##0.000\)"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -41,16 +41,53 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F7FBFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2F0D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF5FB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -73,12 +110,36 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <bottom style="medium">
+        <color rgb="008EA9C1"/>
+      </bottom>
+    </border>
+    <border>
+      <bottom style="thin">
+        <color rgb="00C7D3E0"/>
+      </bottom>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00D9D9D9"/>
+      </left>
+      <right style="thin">
+        <color rgb="00D9D9D9"/>
+      </right>
+      <top style="thin">
+        <color rgb="00D9D9D9"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00D9D9D9"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="42" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
@@ -95,6 +156,73 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
     <xf numFmtId="165" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="2" fontId="2" fillId="6" borderId="3" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="3" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="2" fontId="0" fillId="6" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="42" fontId="3" fillId="2" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="2" fillId="6" borderId="3" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="42" fontId="2" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="3" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="165" fontId="2" fillId="6" borderId="3" pivotButton="0" quotePrefix="0" xfId="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -458,63 +586,72 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="001F4E78"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J49"/>
+  <dimension ref="A1:J81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="35.5703125" customWidth="1" min="1" max="1"/>
-    <col width="15" customWidth="1" min="2" max="2"/>
-    <col width="15.7109375" customWidth="1" min="3" max="3"/>
-    <col width="13.7109375" customWidth="1" min="4" max="4"/>
-    <col width="15.42578125" customWidth="1" min="5" max="5"/>
-    <col width="16.5703125" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="16.85546875" customWidth="1" min="8" max="8"/>
-    <col width="19" bestFit="1" customWidth="1" min="9" max="9"/>
-    <col width="13.140625" bestFit="1" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="22" bestFit="1" customWidth="1" min="9" max="9"/>
+    <col width="19" bestFit="1" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="35" t="inlineStr">
         <is>
           <t>Parameter</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="35" t="inlineStr">
         <is>
           <t>Value</t>
         </is>
       </c>
+      <c r="C1" s="35" t="n"/>
+      <c r="D1" s="35" t="n"/>
+      <c r="E1" s="35" t="n"/>
+      <c r="F1" s="35" t="n"/>
+      <c r="G1" s="35" t="n"/>
+      <c r="H1" s="35" t="n"/>
+      <c r="I1" s="35" t="n"/>
+      <c r="J1" s="35" t="n"/>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="12" t="inlineStr">
         <is>
           <t>Number of Stages</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="13" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>Number of Components</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="13" t="n">
         <v>3</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="12" t="inlineStr">
         <is>
           <t>Condenser Type</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -538,12 +675,12 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="12" t="inlineStr">
         <is>
           <t>Component Name</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>n-Propane</t>
         </is>
@@ -560,808 +697,1170 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="inlineStr">
+      <c r="A7" s="12" t="inlineStr">
         <is>
           <t>Condenser Duty (Btu/h)</t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="13" t="n">
         <v>-49640000</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="inlineStr">
+      <c r="A8" s="12" t="inlineStr">
         <is>
           <t>Reboiler Duty (Btu/h)</t>
         </is>
       </c>
-      <c r="B8" t="n">
+      <c r="B8" s="13" t="n">
         <v>54706000</v>
       </c>
     </row>
+    <row r="9"/>
     <row r="10">
-      <c r="A10" t="inlineStr">
+      <c r="A10" s="12" t="inlineStr">
         <is>
           <t>Simulation Length (min)</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="13" t="n">
         <v>0.00666666</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
+      <c r="A11" s="12" t="inlineStr">
         <is>
           <t>Timestep (sec)</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="13" t="n">
         <v>0.2</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
+      <c r="A12" s="12" t="inlineStr">
         <is>
           <t>Log Frequency (timesteps)</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="13" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>Thermo refresh Delta T (F)</t>
         </is>
       </c>
+      <c r="B13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
+      <c r="A14" s="12" t="inlineStr">
         <is>
           <t>Stage time constant [tau] (sec)</t>
         </is>
       </c>
-      <c r="B14" t="n">
+      <c r="B14" s="13" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr">
+      <c r="A15" s="12" t="inlineStr">
         <is>
           <t>Top Accumulator Holdup (lbmol)</t>
         </is>
       </c>
-      <c r="B15" t="n">
+      <c r="B15" s="13" t="n">
         <v>1388.9</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
+      <c r="A16" s="12" t="inlineStr">
         <is>
           <t>Bottom Holdup (lbmol)</t>
         </is>
       </c>
-      <c r="B16" t="n">
+      <c r="B16" s="13" t="n">
         <v>794</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
+      <c r="A17" s="12" t="inlineStr">
         <is>
           <t>Vapor Holdup Relaxation (sec)</t>
         </is>
       </c>
-      <c r="B17" t="n">
+      <c r="B17" s="13" t="n">
         <v>25</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="inlineStr">
+      <c r="A18" s="12" t="inlineStr">
         <is>
           <t xml:space="preserve">Vapor Flow Relaxation (sec) </t>
         </is>
       </c>
-      <c r="B18" t="n">
+      <c r="B18" s="13" t="n">
         <v>12</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
+      <c r="A19" s="12" t="inlineStr">
         <is>
           <t>Dry Tray K</t>
         </is>
       </c>
-      <c r="B19" t="n">
+      <c r="B19" s="13" t="n">
         <v>40</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="inlineStr">
+      <c r="A20" s="12" t="inlineStr">
         <is>
           <t>Pressure Model</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>Hydraulic</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="inlineStr">
+      <c r="A21" s="12" t="inlineStr">
         <is>
           <t>Vapor Flow Model</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>energy</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" t="inlineStr">
+      <c r="A22" s="12" t="inlineStr">
         <is>
           <t>Condenser Pressure Drop (psi)</t>
         </is>
       </c>
-      <c r="B22" t="n">
+      <c r="B22" s="13" t="n">
         <v>2</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" t="inlineStr">
+      <c r="A23" s="12" t="inlineStr">
         <is>
           <t>Overhead Vapor Line Volume (ft3)</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B23" s="13" t="n">
         <v>56</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" t="inlineStr">
+      <c r="A24" s="12" t="inlineStr">
         <is>
           <t>Condenser Vapor Volume (ft3)</t>
         </is>
       </c>
-      <c r="B24" t="n">
+      <c r="B24" s="13" t="n">
         <v>100</v>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" s="36" t="inlineStr">
+        <is>
+          <t>Operating / Control Defaults</t>
+        </is>
+      </c>
+      <c r="B25" s="37" t="n"/>
+    </row>
     <row r="26">
-      <c r="A26" t="inlineStr">
+      <c r="A26" s="38" t="inlineStr">
+        <is>
+          <t>Enable Level Control</t>
+        </is>
+      </c>
+      <c r="B26" s="38" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="38" t="inlineStr">
+        <is>
+          <t>Top Level PV Mode</t>
+        </is>
+      </c>
+      <c r="B27" s="38" t="inlineStr">
+        <is>
+          <t>true-level</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="39" t="inlineStr">
+        <is>
+          <t>Top Level Kc</t>
+        </is>
+      </c>
+      <c r="B28" s="39" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="39" t="inlineStr">
+        <is>
+          <t>Top Level Ti (sec)</t>
+        </is>
+      </c>
+      <c r="B29" s="39" t="n">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="38" t="inlineStr">
+        <is>
+          <t>Bottom Level PV Mode</t>
+        </is>
+      </c>
+      <c r="B30" s="38" t="inlineStr">
+        <is>
+          <t>true-level</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="39" t="inlineStr">
+        <is>
+          <t>Bottom Level Kc</t>
+        </is>
+      </c>
+      <c r="B31" s="39" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="39" t="inlineStr">
+        <is>
+          <t>Bottom Level Ti (sec)</t>
+        </is>
+      </c>
+      <c r="B32" s="39" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="38" t="inlineStr">
+        <is>
+          <t>Enable Pressure Control</t>
+        </is>
+      </c>
+      <c r="B33" s="38" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="38" t="inlineStr">
+        <is>
+          <t>Pressure Control MV</t>
+        </is>
+      </c>
+      <c r="B34" s="38" t="inlineStr">
+        <is>
+          <t>condenser-duty</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="39" t="inlineStr">
+        <is>
+          <t>Top Pressure SP (psia)</t>
+        </is>
+      </c>
+      <c r="B35" s="39" t="n">
+        <v>220.44</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="39" t="inlineStr">
+        <is>
+          <t>Top Pressure Kc</t>
+        </is>
+      </c>
+      <c r="B36" s="39" t="n">
+        <v>-150000</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="39" t="inlineStr">
+        <is>
+          <t>Top Pressure Ti (sec)</t>
+        </is>
+      </c>
+      <c r="B37" s="39" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="38" t="inlineStr">
+        <is>
+          <t>Equilibrium Relaxation Mode</t>
+        </is>
+      </c>
+      <c r="B38" s="38" t="inlineStr">
+        <is>
+          <t>phase-holdup</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="38" t="inlineStr">
+        <is>
+          <t>Equilibrium Tau (sec)</t>
+        </is>
+      </c>
+      <c r="B39" s="38" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="38" t="inlineStr">
+        <is>
+          <t>Equilibrium Energy Damping Gain</t>
+        </is>
+      </c>
+      <c r="B40" s="38" t="n">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="38" t="inlineStr">
+        <is>
+          <t>Equilibrium Relaxation Live PR</t>
+        </is>
+      </c>
+      <c r="B41" s="38" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="38" t="inlineStr">
+        <is>
+          <t>Enable Distillate Composition Control</t>
+        </is>
+      </c>
+      <c r="B42" s="38" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="39" t="inlineStr">
+        <is>
+          <t>Distillate Composition Component</t>
+        </is>
+      </c>
+      <c r="B43" s="39" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="39" t="inlineStr">
+        <is>
+          <t>Distillate Composition SP</t>
+        </is>
+      </c>
+      <c r="B44" s="39" t="n">
+        <v>0.11</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="39" t="inlineStr">
+        <is>
+          <t>Distillate Composition Kc</t>
+        </is>
+      </c>
+      <c r="B45" s="39" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="39" t="inlineStr">
+        <is>
+          <t>Distillate Composition Ti (sec)</t>
+        </is>
+      </c>
+      <c r="B46" s="39" t="n">
+        <v>600</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="39" t="inlineStr">
+        <is>
+          <t>Distillate Composition Reflux Min (lbmol/h)</t>
+        </is>
+      </c>
+      <c r="B47" s="39" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="39" t="inlineStr">
+        <is>
+          <t>Distillate Composition Reflux Max (lbmol/h)</t>
+        </is>
+      </c>
+      <c r="B48" s="39" t="n">
+        <v>10000</v>
+      </c>
+    </row>
+    <row r="49"/>
+    <row r="50"/>
+    <row r="51">
+      <c r="A51" s="40" t="inlineStr">
         <is>
           <t>Distillate Drum Diameter (ft)</t>
         </is>
       </c>
-      <c r="B26" t="n">
+      <c r="B51" s="41" t="n">
         <v>12.1</v>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="52">
+      <c r="A52" s="40" t="inlineStr">
         <is>
           <t>Distillate Drum Length (ft)</t>
         </is>
       </c>
-      <c r="B27" t="n">
+      <c r="B52" s="41" t="n">
         <v>36.3</v>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
+    <row r="53">
+      <c r="A53" s="40" t="inlineStr">
         <is>
           <t>Distillate Drum Liquid Fraction</t>
         </is>
       </c>
-      <c r="B28" t="n">
+      <c r="B53" s="41" t="n">
         <v>0.5</v>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="40" t="inlineStr">
+        <is>
+          <t>Bottom Sump Diameter (ft)</t>
+        </is>
+      </c>
+      <c r="B54" s="41" t="n">
+        <v>18.1759</v>
+      </c>
+      <c r="C54" s="10" t="n"/>
+      <c r="D54" s="10" t="n"/>
+      <c r="E54" s="10" t="n"/>
+      <c r="F54" s="10" t="n"/>
+      <c r="G54" s="10" t="n"/>
+      <c r="H54" s="10" t="n"/>
+      <c r="I54" s="10" t="n"/>
+      <c r="J54" s="10" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="40" t="inlineStr">
+        <is>
+          <t>Bottom Sump Height (ft)</t>
+        </is>
+      </c>
+      <c r="B55" s="41" t="n">
+        <v>12</v>
+      </c>
+      <c r="C55" s="10" t="n"/>
+      <c r="D55" s="10" t="n"/>
+      <c r="E55" s="10" t="n"/>
+      <c r="F55" s="10" t="n"/>
+      <c r="G55" s="10" t="n"/>
+      <c r="H55" s="10" t="n"/>
+      <c r="I55" s="10" t="n"/>
+      <c r="J55" s="10" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="40" t="inlineStr">
+        <is>
+          <t>Bottom Sump Liquid Fraction</t>
+        </is>
+      </c>
+      <c r="B56" s="41" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C56" s="10" t="n"/>
+      <c r="D56" s="10" t="n"/>
+      <c r="E56" s="10" t="n"/>
+      <c r="F56" s="10" t="n"/>
+      <c r="G56" s="10" t="n"/>
+      <c r="H56" s="10" t="n"/>
+      <c r="I56" s="10" t="n"/>
+      <c r="J56" s="10" t="n"/>
+    </row>
+    <row r="57"/>
+    <row r="58">
+      <c r="A58" s="35" t="inlineStr">
         <is>
           <t>Stage Geometry</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B58" s="35" t="inlineStr">
         <is>
           <t>Start Stage</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr">
+      <c r="C58" s="35" t="inlineStr">
         <is>
           <t>End Stage</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr">
+      <c r="D58" s="35" t="inlineStr">
         <is>
           <t xml:space="preserve">Diameter (ft) </t>
         </is>
       </c>
-      <c r="E30" t="inlineStr">
+      <c r="E58" s="35" t="inlineStr">
         <is>
           <t>Tray Spacing (ft)</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr">
+      <c r="F58" s="11" t="inlineStr">
         <is>
           <t>Gas Void Fraction</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr">
+      <c r="G58" s="11" t="inlineStr">
         <is>
           <t>Weir Height (in)</t>
         </is>
       </c>
-      <c r="H30" t="inlineStr">
+      <c r="H58" s="11" t="inlineStr">
         <is>
           <t>Weir Length (ft)</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr">
+      <c r="I58" s="11" t="inlineStr">
         <is>
           <t>Active Area Fraction</t>
         </is>
       </c>
-      <c r="J30" t="inlineStr">
+      <c r="J58" s="11" t="inlineStr">
         <is>
           <t>System factor</t>
         </is>
       </c>
     </row>
-    <row r="31">
-      <c r="B31" t="n">
+    <row r="59">
+      <c r="B59" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="C31" t="n">
+      <c r="C59" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="D31" t="n">
+      <c r="D59" s="18" t="n">
         <v>16.9619</v>
       </c>
-      <c r="E31" t="n">
+      <c r="E59" s="18" t="n">
         <v>5</v>
       </c>
-      <c r="F31" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G31" t="n">
+      <c r="F59" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G59" s="18" t="n">
         <v>2</v>
       </c>
-      <c r="H31" t="n">
+      <c r="H59" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="I31" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J31" t="n">
+      <c r="I59" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J59" s="18" t="n">
         <v>2.345584585653025</v>
       </c>
     </row>
-    <row r="32">
-      <c r="B32" t="n">
+    <row r="60">
+      <c r="B60" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="C32" t="n">
+      <c r="C60" s="19" t="n">
         <v>3</v>
       </c>
-      <c r="D32" t="n">
+      <c r="D60" s="19" t="n">
         <v>16.9619</v>
       </c>
-      <c r="E32" t="n">
+      <c r="E60" s="19" t="n">
         <v>1.5</v>
       </c>
-      <c r="F32" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G32" t="n">
+      <c r="F60" s="19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G60" s="19" t="n">
         <v>1.65625</v>
       </c>
-      <c r="H32" t="n">
+      <c r="H60" s="19" t="n">
         <v>9</v>
       </c>
-      <c r="I32" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J32" t="n">
+      <c r="I60" s="19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J60" s="19" t="n">
         <v>2.034415244737885</v>
       </c>
     </row>
-    <row r="33">
-      <c r="B33" t="n">
+    <row r="61">
+      <c r="B61" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="C33" t="n">
+      <c r="C61" s="18" t="n">
         <v>4</v>
       </c>
-      <c r="D33" t="n">
+      <c r="D61" s="18" t="n">
         <v>16.9619</v>
       </c>
-      <c r="E33" t="n">
+      <c r="E61" s="18" t="n">
         <v>1.5</v>
       </c>
-      <c r="F33" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G33" t="n">
+      <c r="F61" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G61" s="18" t="n">
         <v>1.65625</v>
       </c>
-      <c r="H33" t="n">
+      <c r="H61" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="I33" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J33" t="n">
+      <c r="I61" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J61" s="18" t="n">
         <v>2.020019101661949</v>
       </c>
     </row>
-    <row r="34">
-      <c r="B34" t="n">
+    <row r="62">
+      <c r="B62" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="C34" t="n">
+      <c r="C62" s="19" t="n">
         <v>5</v>
       </c>
-      <c r="D34" t="n">
+      <c r="D62" s="19" t="n">
         <v>16.9619</v>
       </c>
-      <c r="E34" t="n">
+      <c r="E62" s="19" t="n">
         <v>1.5</v>
       </c>
-      <c r="F34" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G34" t="n">
+      <c r="F62" s="19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G62" s="19" t="n">
         <v>1.65625</v>
       </c>
-      <c r="H34" t="n">
+      <c r="H62" s="19" t="n">
         <v>9</v>
       </c>
-      <c r="I34" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J34" t="n">
+      <c r="I62" s="19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J62" s="19" t="n">
         <v>2.063712381601012</v>
       </c>
     </row>
-    <row r="35">
-      <c r="B35" t="n">
+    <row r="63">
+      <c r="B63" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="C35" t="n">
+      <c r="C63" s="18" t="n">
         <v>6</v>
       </c>
-      <c r="D35" t="n">
+      <c r="D63" s="18" t="n">
         <v>16.9619</v>
       </c>
-      <c r="E35" t="n">
+      <c r="E63" s="18" t="n">
         <v>1.5</v>
       </c>
-      <c r="F35" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G35" t="n">
+      <c r="F63" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G63" s="18" t="n">
         <v>1.65625</v>
       </c>
-      <c r="H35" t="n">
+      <c r="H63" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="I35" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J35" t="n">
+      <c r="I63" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J63" s="18" t="n">
         <v>2.093362957133696</v>
       </c>
     </row>
-    <row r="36">
-      <c r="B36" t="n">
+    <row r="64">
+      <c r="B64" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="C36" t="n">
+      <c r="C64" s="19" t="n">
         <v>7</v>
       </c>
-      <c r="D36" t="n">
+      <c r="D64" s="19" t="n">
         <v>16.9619</v>
       </c>
-      <c r="E36" t="n">
+      <c r="E64" s="19" t="n">
         <v>1.5</v>
       </c>
-      <c r="F36" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G36" t="n">
+      <c r="F64" s="19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G64" s="19" t="n">
         <v>1.65625</v>
       </c>
-      <c r="H36" t="n">
+      <c r="H64" s="19" t="n">
         <v>9</v>
       </c>
-      <c r="I36" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J36" t="n">
+      <c r="I64" s="19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J64" s="19" t="n">
         <v>2.117481801587284</v>
       </c>
     </row>
-    <row r="37">
-      <c r="B37" t="n">
+    <row r="65">
+      <c r="B65" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="C37" t="n">
+      <c r="C65" s="18" t="n">
         <v>8</v>
       </c>
-      <c r="D37" t="n">
+      <c r="D65" s="18" t="n">
         <v>16.9619</v>
       </c>
-      <c r="E37" t="n">
+      <c r="E65" s="18" t="n">
         <v>1.5</v>
       </c>
-      <c r="F37" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G37" t="n">
+      <c r="F65" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G65" s="18" t="n">
         <v>1.65625</v>
       </c>
-      <c r="H37" t="n">
+      <c r="H65" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="I37" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J37" t="n">
+      <c r="I65" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J65" s="18" t="n">
         <v>2.138648585643381</v>
       </c>
     </row>
-    <row r="38">
-      <c r="B38" t="n">
+    <row r="66">
+      <c r="B66" s="19" t="n">
         <v>9</v>
       </c>
-      <c r="C38" t="n">
+      <c r="C66" s="19" t="n">
         <v>9</v>
       </c>
-      <c r="D38" t="n">
+      <c r="D66" s="19" t="n">
         <v>16.9619</v>
       </c>
-      <c r="E38" t="n">
+      <c r="E66" s="19" t="n">
         <v>1.5</v>
       </c>
-      <c r="F38" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G38" t="n">
+      <c r="F66" s="19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G66" s="19" t="n">
         <v>1.65625</v>
       </c>
-      <c r="H38" t="n">
+      <c r="H66" s="19" t="n">
         <v>9</v>
       </c>
-      <c r="I38" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J38" t="n">
+      <c r="I66" s="19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J66" s="19" t="n">
         <v>2.153566343247876</v>
       </c>
     </row>
-    <row r="39">
-      <c r="B39" t="n">
+    <row r="67">
+      <c r="B67" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="C39" t="n">
+      <c r="C67" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="D39" t="n">
+      <c r="D67" s="18" t="n">
         <v>16.9619</v>
       </c>
-      <c r="E39" t="n">
+      <c r="E67" s="18" t="n">
         <v>1.5</v>
       </c>
-      <c r="F39" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G39" t="n">
+      <c r="F67" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G67" s="18" t="n">
         <v>1.65625</v>
       </c>
-      <c r="H39" t="n">
+      <c r="H67" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="I39" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J39" t="n">
+      <c r="I67" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J67" s="18" t="n">
         <v>2.15311883103114</v>
       </c>
     </row>
-    <row r="40">
-      <c r="B40" t="n">
+    <row r="68">
+      <c r="B68" s="19" t="n">
         <v>11</v>
       </c>
-      <c r="C40" t="n">
+      <c r="C68" s="19" t="n">
         <v>11</v>
       </c>
-      <c r="D40" t="n">
+      <c r="D68" s="19" t="n">
         <v>16.9619</v>
       </c>
-      <c r="E40" t="n">
+      <c r="E68" s="19" t="n">
         <v>1.5</v>
       </c>
-      <c r="F40" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G40" t="n">
+      <c r="F68" s="19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G68" s="19" t="n">
         <v>1.65625</v>
       </c>
-      <c r="H40" t="n">
+      <c r="H68" s="19" t="n">
         <v>9</v>
       </c>
-      <c r="I40" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J40" t="n">
+      <c r="I68" s="19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J68" s="19" t="n">
         <v>2.152936458645271</v>
       </c>
     </row>
-    <row r="41">
-      <c r="B41" t="n">
+    <row r="69">
+      <c r="B69" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="C41" t="n">
+      <c r="C69" s="18" t="n">
         <v>12</v>
       </c>
-      <c r="D41" t="n">
+      <c r="D69" s="18" t="n">
         <v>16.9619</v>
       </c>
-      <c r="E41" t="n">
+      <c r="E69" s="18" t="n">
         <v>1.5</v>
       </c>
-      <c r="F41" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G41" t="n">
+      <c r="F69" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G69" s="18" t="n">
         <v>1.65625</v>
       </c>
-      <c r="H41" t="n">
+      <c r="H69" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="I41" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J41" t="n">
+      <c r="I69" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J69" s="18" t="n">
         <v>1.343361485962905</v>
       </c>
     </row>
-    <row r="42">
-      <c r="B42" t="n">
+    <row r="70">
+      <c r="B70" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="C42" t="n">
+      <c r="C70" s="19" t="n">
         <v>13</v>
       </c>
-      <c r="D42" t="n">
+      <c r="D70" s="19" t="n">
         <v>16.9619</v>
       </c>
-      <c r="E42" t="n">
+      <c r="E70" s="19" t="n">
         <v>1.5</v>
       </c>
-      <c r="F42" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G42" t="n">
+      <c r="F70" s="19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G70" s="19" t="n">
         <v>1.65625</v>
       </c>
-      <c r="H42" t="n">
+      <c r="H70" s="19" t="n">
         <v>9</v>
       </c>
-      <c r="I42" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J42" t="n">
+      <c r="I70" s="19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J70" s="19" t="n">
         <v>1.351651678029181</v>
       </c>
     </row>
-    <row r="43">
-      <c r="B43" t="n">
+    <row r="71">
+      <c r="B71" s="18" t="n">
         <v>14</v>
       </c>
-      <c r="C43" t="n">
+      <c r="C71" s="18" t="n">
         <v>14</v>
       </c>
-      <c r="D43" t="n">
+      <c r="D71" s="18" t="n">
         <v>16.9619</v>
       </c>
-      <c r="E43" t="n">
+      <c r="E71" s="18" t="n">
         <v>1.5</v>
       </c>
-      <c r="F43" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G43" t="n">
+      <c r="F71" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G71" s="18" t="n">
         <v>1.65625</v>
       </c>
-      <c r="H43" t="n">
+      <c r="H71" s="18" t="n">
         <v>9</v>
       </c>
-      <c r="I43" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J43" t="n">
+      <c r="I71" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J71" s="18" t="n">
         <v>1.360189094835164</v>
       </c>
     </row>
-    <row r="44">
-      <c r="B44" t="n">
+    <row r="72">
+      <c r="B72" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="C44" t="n">
+      <c r="C72" s="19" t="n">
         <v>15</v>
       </c>
-      <c r="D44" t="n">
+      <c r="D72" s="19" t="n">
         <v>16.9619</v>
       </c>
-      <c r="E44" t="n">
+      <c r="E72" s="19" t="n">
         <v>1.5</v>
       </c>
-      <c r="F44" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G44" t="n">
+      <c r="F72" s="19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G72" s="19" t="n">
         <v>1.65625</v>
       </c>
-      <c r="H44" t="n">
+      <c r="H72" s="19" t="n">
         <v>9</v>
       </c>
-      <c r="I44" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J44" t="n">
+      <c r="I72" s="19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J72" s="19" t="n">
         <v>1.3233022940368</v>
       </c>
     </row>
-    <row r="45">
-      <c r="B45" t="n">
+    <row r="73">
+      <c r="B73" s="18" t="n">
         <v>16</v>
       </c>
-      <c r="C45" t="n">
+      <c r="C73" s="18" t="n">
         <v>16</v>
       </c>
-      <c r="D45" t="n">
+      <c r="D73" s="18" t="n">
         <v>18.1759</v>
       </c>
-      <c r="E45" t="n">
+      <c r="E73" s="18" t="n">
         <v>1.5</v>
       </c>
-      <c r="F45" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G45" t="n">
+      <c r="F73" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G73" s="18" t="n">
         <v>1.98125</v>
       </c>
-      <c r="H45" t="n">
+      <c r="H73" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="I45" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J45" t="n">
+      <c r="I73" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J73" s="18" t="n">
         <v>1.290881129536785</v>
       </c>
     </row>
-    <row r="46">
-      <c r="B46" t="n">
+    <row r="74">
+      <c r="B74" s="19" t="n">
         <v>17</v>
       </c>
-      <c r="C46" t="n">
+      <c r="C74" s="19" t="n">
         <v>17</v>
       </c>
-      <c r="D46" t="n">
+      <c r="D74" s="19" t="n">
         <v>18.1759</v>
       </c>
-      <c r="E46" t="n">
+      <c r="E74" s="19" t="n">
         <v>1.5</v>
       </c>
-      <c r="F46" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G46" t="n">
+      <c r="F74" s="19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G74" s="19" t="n">
         <v>1.98125</v>
       </c>
-      <c r="H46" t="n">
+      <c r="H74" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="I46" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J46" t="n">
+      <c r="I74" s="19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J74" s="19" t="n">
         <v>1.298200448928769</v>
       </c>
     </row>
-    <row r="47">
-      <c r="B47" t="n">
+    <row r="75">
+      <c r="B75" s="18" t="n">
         <v>18</v>
       </c>
-      <c r="C47" t="n">
+      <c r="C75" s="18" t="n">
         <v>18</v>
       </c>
-      <c r="D47" t="n">
+      <c r="D75" s="18" t="n">
         <v>18.1759</v>
       </c>
-      <c r="E47" t="n">
+      <c r="E75" s="18" t="n">
         <v>1.5</v>
       </c>
-      <c r="F47" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G47" t="n">
+      <c r="F75" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G75" s="18" t="n">
         <v>1.98125</v>
       </c>
-      <c r="H47" t="n">
+      <c r="H75" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="I47" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J47" t="n">
+      <c r="I75" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J75" s="18" t="n">
         <v>1.451809993105148</v>
       </c>
     </row>
-    <row r="48">
-      <c r="B48" t="n">
+    <row r="76">
+      <c r="B76" s="19" t="n">
         <v>19</v>
       </c>
-      <c r="C48" t="n">
+      <c r="C76" s="19" t="n">
         <v>19</v>
       </c>
-      <c r="D48" t="n">
+      <c r="D76" s="19" t="n">
         <v>18.1759</v>
       </c>
-      <c r="E48" t="n">
+      <c r="E76" s="19" t="n">
         <v>1.5</v>
       </c>
-      <c r="F48" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G48" t="n">
+      <c r="F76" s="19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G76" s="19" t="n">
         <v>1.98125</v>
       </c>
-      <c r="H48" t="n">
+      <c r="H76" s="19" t="n">
         <v>10</v>
       </c>
-      <c r="I48" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J48" t="n">
+      <c r="I76" s="19" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J76" s="19" t="n">
         <v>1.421500730346922</v>
       </c>
     </row>
-    <row r="49">
-      <c r="B49" t="n">
+    <row r="77">
+      <c r="B77" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="C49" t="n">
+      <c r="C77" s="18" t="n">
         <v>20</v>
       </c>
-      <c r="D49" t="n">
+      <c r="D77" s="18" t="n">
         <v>18.1759</v>
       </c>
-      <c r="E49" t="n">
+      <c r="E77" s="18" t="n">
         <v>1.5</v>
       </c>
-      <c r="F49" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="G49" t="n">
+      <c r="F77" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="G77" s="18" t="n">
         <v>1.98125</v>
       </c>
-      <c r="H49" t="n">
+      <c r="H77" s="18" t="n">
         <v>10</v>
       </c>
-      <c r="I49" t="n">
-        <v>0.75</v>
-      </c>
-      <c r="J49" t="n">
+      <c r="I77" s="18" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="J77" s="18" t="n">
         <v>1</v>
       </c>
+    </row>
+    <row r="78"/>
+    <row r="79">
+      <c r="A79" s="40" t="inlineStr">
+        <is>
+          <t>Bottom Sump Diameter (ft)</t>
+        </is>
+      </c>
+      <c r="B79" s="41" t="n">
+        <v>18.1759</v>
+      </c>
+      <c r="C79" s="18" t="n"/>
+      <c r="D79" s="18" t="n"/>
+      <c r="E79" s="18" t="n"/>
+      <c r="F79" s="18" t="n"/>
+      <c r="G79" s="18" t="n"/>
+      <c r="H79" s="18" t="n"/>
+      <c r="I79" s="18" t="n"/>
+      <c r="J79" s="18" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="40" t="inlineStr">
+        <is>
+          <t>Bottom Sump height (ft)</t>
+        </is>
+      </c>
+      <c r="B80" s="42" t="n">
+        <v>12</v>
+      </c>
+      <c r="C80" s="19" t="n"/>
+      <c r="D80" s="19" t="n"/>
+      <c r="E80" s="19" t="n"/>
+      <c r="F80" s="19" t="n"/>
+      <c r="G80" s="19" t="n"/>
+      <c r="H80" s="19" t="n"/>
+      <c r="I80" s="19" t="n"/>
+      <c r="J80" s="19" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="40" t="inlineStr">
+        <is>
+          <t>Bottom Sump Liquid Fraction</t>
+        </is>
+      </c>
+      <c r="B81" s="41" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="C81" s="18" t="n"/>
+      <c r="D81" s="18" t="n"/>
+      <c r="E81" s="18" t="n"/>
+      <c r="F81" s="18" t="n"/>
+      <c r="G81" s="18" t="n"/>
+      <c r="H81" s="18" t="n"/>
+      <c r="I81" s="18" t="n"/>
+      <c r="J81" s="18" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1371,841 +1870,846 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="005B9BD5"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:L21"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="34.28515625" defaultRowHeight="15"/>
   <cols>
-    <col width="5.85546875" bestFit="1" customWidth="1" min="1" max="1"/>
-    <col width="15.5703125" bestFit="1" customWidth="1" style="3" min="2" max="2"/>
-    <col width="14.28515625" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
-    <col width="20.28515625" bestFit="1" customWidth="1" style="3" min="4" max="4"/>
-    <col width="20.42578125" bestFit="1" customWidth="1" style="3" min="5" max="5"/>
-    <col width="20.5703125" bestFit="1" customWidth="1" min="6" max="6"/>
-    <col width="31" bestFit="1" customWidth="1" style="7" min="7" max="9"/>
-    <col width="31.140625" bestFit="1" customWidth="1" style="7" min="10" max="12"/>
+    <col width="10" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="17" bestFit="1" customWidth="1" style="3" min="2" max="2"/>
+    <col width="17" bestFit="1" customWidth="1" style="3" min="3" max="3"/>
+    <col width="22" bestFit="1" customWidth="1" style="3" min="4" max="4"/>
+    <col width="23" bestFit="1" customWidth="1" style="3" min="5" max="5"/>
+    <col width="23" bestFit="1" customWidth="1" min="6" max="6"/>
+    <col width="28" bestFit="1" customWidth="1" style="7" min="7" max="9"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="28" bestFit="1" customWidth="1" style="7" min="10" max="12"/>
+    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="11" t="inlineStr">
         <is>
           <t>Stage</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="21" t="inlineStr">
         <is>
           <t>Temperature (F)</t>
         </is>
       </c>
-      <c r="C1" s="4" t="inlineStr">
+      <c r="C1" s="21" t="inlineStr">
         <is>
           <t>Pressure (psia)</t>
         </is>
       </c>
-      <c r="D1" s="4" t="inlineStr">
+      <c r="D1" s="21" t="inlineStr">
         <is>
           <t>Vapor Flow (lbmol/h)</t>
         </is>
       </c>
-      <c r="E1" s="4" t="inlineStr">
+      <c r="E1" s="21" t="inlineStr">
         <is>
           <t>Liquid Flow (lbmol/h)</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="11" t="inlineStr">
         <is>
           <t>Liquid Holdup (lbmol)</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="G1" s="22" t="inlineStr">
         <is>
           <t>Vapor Composition Component 1</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="H1" s="22" t="inlineStr">
         <is>
           <t>Vapor Composition Component 2</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="I1" s="22" t="inlineStr">
         <is>
           <t>Vapor Composition Component 3</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="J1" s="22" t="inlineStr">
         <is>
           <t>Liquid Composition Component 1</t>
         </is>
       </c>
-      <c r="K1" s="6" t="inlineStr">
+      <c r="K1" s="22" t="inlineStr">
         <is>
           <t>Liquid Composition Component 2</t>
         </is>
       </c>
-      <c r="L1" s="6" t="inlineStr">
+      <c r="L1" s="22" t="inlineStr">
         <is>
           <t>Liquid Composition Component 3</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="n">
+      <c r="A2" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="B2" s="5" t="n">
+      <c r="B2" s="23" t="n">
         <v>118.742</v>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="23" t="n">
         <v>220.44</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="24" t="n">
         <v>0</v>
       </c>
-      <c r="E2" s="5" t="n">
+      <c r="E2" s="23" t="n">
         <v>5952.48</v>
       </c>
-      <c r="F2" t="n">
+      <c r="F2" s="13" t="n">
         <v>0</v>
       </c>
-      <c r="G2" s="8" t="n">
+      <c r="G2" s="25" t="n">
         <v>0.958851</v>
       </c>
-      <c r="H2" s="8" t="n">
+      <c r="H2" s="25" t="n">
         <v>0.041148</v>
       </c>
-      <c r="I2" s="8" t="n">
+      <c r="I2" s="25" t="n">
         <v>1.0753e-06</v>
       </c>
-      <c r="J2" s="8" t="n">
+      <c r="J2" s="25" t="n">
         <v>0.904861</v>
       </c>
-      <c r="K2" s="8" t="n">
+      <c r="K2" s="25" t="n">
         <v>0.09513290000000001</v>
       </c>
-      <c r="L2" s="8" t="n">
+      <c r="L2" s="25" t="n">
         <v>5.9089e-06</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="n">
+      <c r="A3" s="26" t="n">
         <v>2</v>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B3" s="27" t="n">
         <v>126.824</v>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="27" t="n">
         <v>220.44</v>
       </c>
-      <c r="D3" s="5" t="n">
+      <c r="D3" s="27" t="n">
         <v>8333.469999999999</v>
       </c>
-      <c r="E3" s="5" t="n">
+      <c r="E3" s="27" t="n">
         <v>5676.41</v>
       </c>
-      <c r="F3" t="n">
+      <c r="F3" s="26" t="n">
         <v>38.19260297324073</v>
       </c>
-      <c r="G3" s="8" t="n">
+      <c r="G3" s="28" t="n">
         <v>0.904861</v>
       </c>
-      <c r="H3" s="8" t="n">
+      <c r="H3" s="28" t="n">
         <v>0.09513290000000001</v>
       </c>
-      <c r="I3" s="8" t="n">
+      <c r="I3" s="28" t="n">
         <v>5.9089e-06</v>
       </c>
-      <c r="J3" s="8" t="n">
+      <c r="J3" s="28" t="n">
         <v>0.797845</v>
       </c>
-      <c r="K3" s="8" t="n">
+      <c r="K3" s="28" t="n">
         <v>0.202126</v>
       </c>
-      <c r="L3" s="8" t="n">
+      <c r="L3" s="28" t="n">
         <v>2.9338e-05</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="n">
+      <c r="A4" s="13" t="n">
         <v>3</v>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="23" t="n">
         <v>137.246</v>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="23" t="n">
         <v>221.085</v>
       </c>
-      <c r="D4" s="5" t="n">
+      <c r="D4" s="23" t="n">
         <v>8057.4</v>
       </c>
-      <c r="E4" s="5" t="n">
+      <c r="E4" s="23" t="n">
         <v>5450.6</v>
       </c>
-      <c r="F4" t="n">
+      <c r="F4" s="13" t="n">
         <v>34.5146398660006</v>
       </c>
-      <c r="G4" s="8" t="n">
+      <c r="G4" s="25" t="n">
         <v>0.829469</v>
       </c>
-      <c r="H4" s="8" t="n">
+      <c r="H4" s="25" t="n">
         <v>0.170509</v>
       </c>
-      <c r="I4" s="8" t="n">
+      <c r="I4" s="25" t="n">
         <v>2.2414e-05</v>
       </c>
-      <c r="J4" s="8" t="n">
+      <c r="J4" s="25" t="n">
         <v>0.673822</v>
       </c>
-      <c r="K4" s="8" t="n">
+      <c r="K4" s="25" t="n">
         <v>0.326081</v>
       </c>
-      <c r="L4" s="8" t="n">
+      <c r="L4" s="25" t="n">
         <v>9.7855e-05</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="n">
+      <c r="A5" s="26" t="n">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="27" t="n">
         <v>147.812</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="27" t="n">
         <v>221.731</v>
       </c>
-      <c r="D5" s="5" t="n">
+      <c r="D5" s="27" t="n">
         <v>7831.59</v>
       </c>
-      <c r="E5" s="5" t="n">
+      <c r="E5" s="27" t="n">
         <v>5308.06</v>
       </c>
-      <c r="F5" t="n">
+      <c r="F5" s="26" t="n">
         <v>33.46631100031247</v>
       </c>
-      <c r="G5" s="8" t="n">
+      <c r="G5" s="28" t="n">
         <v>0.744063</v>
       </c>
-      <c r="H5" s="8" t="n">
+      <c r="H5" s="28" t="n">
         <v>0.255867</v>
       </c>
-      <c r="I5" s="8" t="n">
+      <c r="I5" s="28" t="n">
         <v>6.990099999999999e-05</v>
       </c>
-      <c r="J5" s="8" t="n">
+      <c r="J5" s="28" t="n">
         <v>0.558525</v>
       </c>
-      <c r="K5" s="8" t="n">
+      <c r="K5" s="28" t="n">
         <v>0.441206</v>
       </c>
-      <c r="L5" s="8" t="n">
+      <c r="L5" s="28" t="n">
         <v>0.00026852</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="n">
+      <c r="A6" s="13" t="n">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="23" t="n">
         <v>156.686</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="23" t="n">
         <v>222.377</v>
       </c>
-      <c r="D6" s="5" t="n">
+      <c r="D6" s="23" t="n">
         <v>7689.05</v>
       </c>
-      <c r="E6" s="5" t="n">
+      <c r="E6" s="23" t="n">
         <v>5237.95</v>
       </c>
-      <c r="F6" t="n">
+      <c r="F6" s="13" t="n">
         <v>32.51477868945729</v>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="G6" s="25" t="n">
         <v>0.665772</v>
       </c>
-      <c r="H6" s="8" t="n">
+      <c r="H6" s="25" t="n">
         <v>0.334041</v>
       </c>
-      <c r="I6" s="8" t="n">
+      <c r="I6" s="25" t="n">
         <v>0.0001872</v>
       </c>
-      <c r="J6" s="8" t="n">
+      <c r="J6" s="25" t="n">
         <v>0.469497</v>
       </c>
-      <c r="K6" s="8" t="n">
+      <c r="K6" s="25" t="n">
         <v>0.529855</v>
       </c>
-      <c r="L6" s="8" t="n">
+      <c r="L6" s="25" t="n">
         <v>0.00064787</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" t="n">
+      <c r="A7" s="26" t="n">
         <v>6</v>
       </c>
-      <c r="B7" s="5" t="n">
+      <c r="B7" s="27" t="n">
         <v>163.13</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="27" t="n">
         <v>223.022</v>
       </c>
-      <c r="D7" s="5" t="n">
+      <c r="D7" s="27" t="n">
         <v>7618.95</v>
       </c>
-      <c r="E7" s="5" t="n">
+      <c r="E7" s="27" t="n">
         <v>5208.97</v>
       </c>
-      <c r="F7" t="n">
+      <c r="F7" s="26" t="n">
         <v>31.89162313823113</v>
       </c>
-      <c r="G7" s="8" t="n">
+      <c r="G7" s="28" t="n">
         <v>0.605553</v>
       </c>
-      <c r="H7" s="8" t="n">
+      <c r="H7" s="28" t="n">
         <v>0.394</v>
       </c>
-      <c r="I7" s="8" t="n">
+      <c r="I7" s="28" t="n">
         <v>0.00044725</v>
       </c>
-      <c r="J7" s="8" t="n">
+      <c r="J7" s="28" t="n">
         <v>0.409112</v>
       </c>
-      <c r="K7" s="8" t="n">
+      <c r="K7" s="28" t="n">
         <v>0.58945</v>
       </c>
-      <c r="L7" s="8" t="n">
+      <c r="L7" s="28" t="n">
         <v>0.00143759</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" t="n">
+      <c r="A8" s="13" t="n">
         <v>7</v>
       </c>
-      <c r="B8" s="5" t="n">
+      <c r="B8" s="23" t="n">
         <v>167.486</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="23" t="n">
         <v>223.668</v>
       </c>
-      <c r="D8" s="5" t="n">
+      <c r="D8" s="23" t="n">
         <v>7589.96</v>
       </c>
-      <c r="E8" s="5" t="n">
+      <c r="E8" s="23" t="n">
         <v>5196.3</v>
       </c>
-      <c r="F8" t="n">
+      <c r="F8" s="13" t="n">
         <v>31.44034629518334</v>
       </c>
-      <c r="G8" s="8" t="n">
+      <c r="G8" s="25" t="n">
         <v>0.56463</v>
       </c>
-      <c r="H8" s="8" t="n">
+      <c r="H8" s="25" t="n">
         <v>0.434382</v>
       </c>
-      <c r="I8" s="8" t="n">
+      <c r="I8" s="25" t="n">
         <v>0.00098846</v>
       </c>
-      <c r="J8" s="8" t="n">
+      <c r="J8" s="25" t="n">
         <v>0.371246</v>
       </c>
-      <c r="K8" s="8" t="n">
+      <c r="K8" s="25" t="n">
         <v>0.625727</v>
       </c>
-      <c r="L8" s="8" t="n">
+      <c r="L8" s="25" t="n">
         <v>0.00302716</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" t="n">
+      <c r="A9" s="26" t="n">
         <v>8</v>
       </c>
-      <c r="B9" s="5" t="n">
+      <c r="B9" s="27" t="n">
         <v>170.366</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="27" t="n">
         <v>224.313</v>
       </c>
-      <c r="D9" s="5" t="n">
+      <c r="D9" s="27" t="n">
         <v>7577.29</v>
       </c>
-      <c r="E9" s="5" t="n">
+      <c r="E9" s="27" t="n">
         <v>5185.3</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F9" s="26" t="n">
         <v>31.13922641427964</v>
       </c>
-      <c r="G9" s="8" t="n">
+      <c r="G9" s="28" t="n">
         <v>0.538922</v>
       </c>
-      <c r="H9" s="8" t="n">
+      <c r="H9" s="28" t="n">
         <v>0.459</v>
       </c>
-      <c r="I9" s="8" t="n">
+      <c r="I9" s="28" t="n">
         <v>0.0020778</v>
       </c>
-      <c r="J9" s="8" t="n">
+      <c r="J9" s="28" t="n">
         <v>0.348396</v>
       </c>
-      <c r="K9" s="8" t="n">
+      <c r="K9" s="28" t="n">
         <v>0.645436</v>
       </c>
-      <c r="L9" s="8" t="n">
+      <c r="L9" s="28" t="n">
         <v>0.00616782</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" t="n">
+      <c r="A10" s="13" t="n">
         <v>9</v>
       </c>
-      <c r="B10" s="5" t="n">
+      <c r="B10" s="23" t="n">
         <v>172.454</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="23" t="n">
         <v>224.959</v>
       </c>
-      <c r="D10" s="5" t="n">
+      <c r="D10" s="23" t="n">
         <v>7566.3</v>
       </c>
-      <c r="E10" s="5" t="n">
+      <c r="E10" s="23" t="n">
         <v>5165.98</v>
       </c>
-      <c r="F10" t="n">
+      <c r="F10" s="13" t="n">
         <v>30.90790274479952</v>
       </c>
-      <c r="G10" s="8" t="n">
+      <c r="G10" s="25" t="n">
         <v>0.5235069999999999</v>
       </c>
-      <c r="H10" s="8" t="n">
+      <c r="H10" s="25" t="n">
         <v>0.472264</v>
       </c>
-      <c r="I10" s="8" t="n">
+      <c r="I10" s="25" t="n">
         <v>0.00422877</v>
       </c>
-      <c r="J10" s="8" t="n">
+      <c r="J10" s="25" t="n">
         <v>0.334565</v>
       </c>
-      <c r="K10" s="8" t="n">
+      <c r="K10" s="25" t="n">
         <v>0.653151</v>
       </c>
-      <c r="L10" s="8" t="n">
+      <c r="L10" s="25" t="n">
         <v>0.0122841</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="n">
+      <c r="A11" s="26" t="n">
         <v>10</v>
       </c>
-      <c r="B11" s="5" t="n">
+      <c r="B11" s="27" t="n">
         <v>174.29</v>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="27" t="n">
         <v>225.605</v>
       </c>
-      <c r="D11" s="5" t="n">
+      <c r="D11" s="27" t="n">
         <v>7546.97</v>
       </c>
-      <c r="E11" s="5" t="n">
+      <c r="E11" s="27" t="n">
         <v>5127.78</v>
       </c>
-      <c r="F11" t="n">
+      <c r="F11" s="26" t="n">
         <v>30.67035248740331</v>
       </c>
-      <c r="G11" s="8" t="n">
+      <c r="G11" s="28" t="n">
         <v>0.5144879999999999</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="H11" s="28" t="n">
         <v>0.477102</v>
       </c>
-      <c r="I11" s="8" t="n">
+      <c r="I11" s="28" t="n">
         <v>0.00841044</v>
       </c>
-      <c r="J11" s="8" t="n">
+      <c r="J11" s="28" t="n">
         <v>0.32552</v>
       </c>
-      <c r="K11" s="8" t="n">
+      <c r="K11" s="28" t="n">
         <v>0.650496</v>
       </c>
-      <c r="L11" s="8" t="n">
+      <c r="L11" s="28" t="n">
         <v>0.0239846</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="n">
+      <c r="A12" s="13" t="n">
         <v>11</v>
       </c>
-      <c r="B12" s="5" t="n">
+      <c r="B12" s="23" t="n">
         <v>176.468</v>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="23" t="n">
         <v>226.25</v>
       </c>
-      <c r="D12" s="5" t="n">
+      <c r="D12" s="23" t="n">
         <v>7508.77</v>
       </c>
-      <c r="E12" s="5" t="n">
+      <c r="E12" s="23" t="n">
         <v>5057.12</v>
       </c>
-      <c r="F12" t="n">
+      <c r="F12" s="13" t="n">
         <v>30.34277233147372</v>
       </c>
-      <c r="G12" s="8" t="n">
+      <c r="G12" s="25" t="n">
         <v>0.509226</v>
       </c>
-      <c r="H12" s="8" t="n">
+      <c r="H12" s="25" t="n">
         <v>0.474393</v>
       </c>
-      <c r="I12" s="8" t="n">
+      <c r="I12" s="25" t="n">
         <v>0.0163811</v>
       </c>
-      <c r="J12" s="8" t="n">
+      <c r="J12" s="25" t="n">
         <v>0.318231</v>
       </c>
-      <c r="K12" s="8" t="n">
+      <c r="K12" s="25" t="n">
         <v>0.636034</v>
       </c>
-      <c r="L12" s="8" t="n">
+      <c r="L12" s="25" t="n">
         <v>0.0457348</v>
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="n">
+      <c r="A13" s="26" t="n">
         <v>12</v>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B13" s="27" t="n">
         <v>179.618</v>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="27" t="n">
         <v>226.896</v>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D13" s="27" t="n">
         <v>7438.11</v>
       </c>
-      <c r="E13" s="5" t="n">
+      <c r="E13" s="27" t="n">
         <v>12352.5</v>
       </c>
-      <c r="F13" t="n">
+      <c r="F13" s="26" t="n">
         <v>51.06214131827053</v>
       </c>
-      <c r="G13" s="8" t="n">
+      <c r="G13" s="28" t="n">
         <v>0.506015</v>
       </c>
-      <c r="H13" s="8" t="n">
+      <c r="H13" s="28" t="n">
         <v>0.462888</v>
       </c>
-      <c r="I13" s="8" t="n">
+      <c r="I13" s="28" t="n">
         <v>0.0310966</v>
       </c>
-      <c r="J13" s="8" t="n">
+      <c r="J13" s="28" t="n">
         <v>0.310303</v>
       </c>
-      <c r="K13" s="8" t="n">
+      <c r="K13" s="28" t="n">
         <v>0.605483</v>
       </c>
-      <c r="L13" s="8" t="n">
+      <c r="L13" s="28" t="n">
         <v>0.08421430000000001</v>
       </c>
     </row>
     <row r="14">
-      <c r="A14" t="n">
+      <c r="A14" s="13" t="n">
         <v>13</v>
       </c>
-      <c r="B14" s="5" t="n">
+      <c r="B14" s="23" t="n">
         <v>182.732</v>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C14" s="23" t="n">
         <v>227.541</v>
       </c>
-      <c r="D14" s="5" t="n">
+      <c r="D14" s="23" t="n">
         <v>7590.51</v>
       </c>
-      <c r="E14" s="5" t="n">
+      <c r="E14" s="23" t="n">
         <v>12382.7</v>
       </c>
-      <c r="F14" t="n">
+      <c r="F14" s="13" t="n">
         <v>50.71399050987867</v>
       </c>
-      <c r="G14" s="8" t="n">
+      <c r="G14" s="25" t="n">
         <v>0.475131</v>
       </c>
-      <c r="H14" s="8" t="n">
+      <c r="H14" s="25" t="n">
         <v>0.49238</v>
       </c>
-      <c r="I14" s="8" t="n">
+      <c r="I14" s="25" t="n">
         <v>0.0324888</v>
       </c>
-      <c r="J14" s="8" t="n">
+      <c r="J14" s="25" t="n">
         <v>0.286487</v>
       </c>
-      <c r="K14" s="8" t="n">
+      <c r="K14" s="25" t="n">
         <v>0.628333</v>
       </c>
-      <c r="L14" s="8" t="n">
+      <c r="L14" s="25" t="n">
         <v>0.08518000000000001</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" t="n">
+      <c r="A15" s="26" t="n">
         <v>14</v>
       </c>
-      <c r="B15" s="5" t="n">
+      <c r="B15" s="27" t="n">
         <v>186.548</v>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C15" s="27" t="n">
         <v>228.187</v>
       </c>
-      <c r="D15" s="5" t="n">
+      <c r="D15" s="27" t="n">
         <v>7620.72</v>
       </c>
-      <c r="E15" s="5" t="n">
+      <c r="E15" s="27" t="n">
         <v>12425.5</v>
       </c>
-      <c r="F15" t="n">
+      <c r="F15" s="26" t="n">
         <v>50.38780860188388</v>
       </c>
-      <c r="G15" s="8" t="n">
+      <c r="G15" s="28" t="n">
         <v>0.43578</v>
       </c>
-      <c r="H15" s="8" t="n">
+      <c r="H15" s="28" t="n">
         <v>0.529957</v>
       </c>
-      <c r="I15" s="8" t="n">
+      <c r="I15" s="28" t="n">
         <v>0.0342629</v>
       </c>
-      <c r="J15" s="8" t="n">
+      <c r="J15" s="28" t="n">
         <v>0.257399</v>
       </c>
-      <c r="K15" s="8" t="n">
+      <c r="K15" s="28" t="n">
         <v>0.656237</v>
       </c>
-      <c r="L15" s="8" t="n">
+      <c r="L15" s="28" t="n">
         <v>0.0863647</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" t="n">
+      <c r="A16" s="13" t="n">
         <v>15</v>
       </c>
-      <c r="B16" s="5" t="n">
+      <c r="B16" s="23" t="n">
         <v>191.012</v>
       </c>
-      <c r="C16" s="5" t="n">
+      <c r="C16" s="23" t="n">
         <v>228.832</v>
       </c>
-      <c r="D16" s="5" t="n">
+      <c r="D16" s="23" t="n">
         <v>7663.52</v>
       </c>
-      <c r="E16" s="5" t="n">
+      <c r="E16" s="23" t="n">
         <v>12485.2</v>
       </c>
-      <c r="F16" t="n">
+      <c r="F16" s="13" t="n">
         <v>51.82777876770178</v>
       </c>
-      <c r="G16" s="8" t="n">
+      <c r="G16" s="25" t="n">
         <v>0.387783</v>
       </c>
-      <c r="H16" s="8" t="n">
+      <c r="H16" s="25" t="n">
         <v>0.575749</v>
       </c>
-      <c r="I16" s="8" t="n">
+      <c r="I16" s="25" t="n">
         <v>0.0364683</v>
       </c>
-      <c r="J16" s="8" t="n">
+      <c r="J16" s="25" t="n">
         <v>0.223657</v>
       </c>
-      <c r="K16" s="8" t="n">
+      <c r="K16" s="25" t="n">
         <v>0.68852</v>
       </c>
-      <c r="L16" s="8" t="n">
+      <c r="L16" s="25" t="n">
         <v>0.08782379999999999</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="n">
+      <c r="A17" s="26" t="n">
         <v>16</v>
       </c>
-      <c r="B17" s="5" t="n">
+      <c r="B17" s="27" t="n">
         <v>196.016</v>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C17" s="27" t="n">
         <v>229.478</v>
       </c>
-      <c r="D17" s="5" t="n">
+      <c r="D17" s="27" t="n">
         <v>7723.22</v>
       </c>
-      <c r="E17" s="5" t="n">
+      <c r="E17" s="27" t="n">
         <v>12563.2</v>
       </c>
-      <c r="F17" t="n">
+      <c r="F17" s="26" t="n">
         <v>62.53531141217334</v>
       </c>
-      <c r="G17" s="8" t="n">
+      <c r="G17" s="28" t="n">
         <v>0.332229</v>
       </c>
-      <c r="H17" s="8" t="n">
+      <c r="H17" s="28" t="n">
         <v>0.628559</v>
       </c>
-      <c r="I17" s="8" t="n">
+      <c r="I17" s="28" t="n">
         <v>0.0392126</v>
       </c>
-      <c r="J17" s="8" t="n">
+      <c r="J17" s="28" t="n">
         <v>0.186706</v>
       </c>
-      <c r="K17" s="8" t="n">
+      <c r="K17" s="28" t="n">
         <v>0.723484</v>
       </c>
-      <c r="L17" s="8" t="n">
+      <c r="L17" s="28" t="n">
         <v>0.0898098</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" t="n">
+      <c r="A18" s="13" t="n">
         <v>17</v>
       </c>
-      <c r="B18" s="5" t="n">
+      <c r="B18" s="23" t="n">
         <v>201.362</v>
       </c>
-      <c r="C18" s="5" t="n">
+      <c r="C18" s="23" t="n">
         <v>230.124</v>
       </c>
-      <c r="D18" s="5" t="n">
+      <c r="D18" s="23" t="n">
         <v>7801.2</v>
       </c>
-      <c r="E18" s="5" t="n">
+      <c r="E18" s="23" t="n">
         <v>12653.8</v>
       </c>
-      <c r="F18" t="n">
+      <c r="F18" s="13" t="n">
         <v>63.86627868425875</v>
       </c>
-      <c r="G18" s="8" t="n">
+      <c r="G18" s="25" t="n">
         <v>0.271637</v>
       </c>
-      <c r="H18" s="8" t="n">
+      <c r="H18" s="25" t="n">
         <v>0.685466</v>
       </c>
-      <c r="I18" s="8" t="n">
+      <c r="I18" s="25" t="n">
         <v>0.0428969</v>
       </c>
-      <c r="J18" s="8" t="n">
+      <c r="J18" s="25" t="n">
         <v>0.148614</v>
       </c>
-      <c r="K18" s="8" t="n">
+      <c r="K18" s="25" t="n">
         <v>0.758166</v>
       </c>
-      <c r="L18" s="8" t="n">
+      <c r="L18" s="25" t="n">
         <v>0.0932195</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="n">
+      <c r="A19" s="26" t="n">
         <v>18</v>
       </c>
-      <c r="B19" s="5" t="n">
+      <c r="B19" s="27" t="n">
         <v>206.942</v>
       </c>
-      <c r="C19" s="5" t="n">
+      <c r="C19" s="27" t="n">
         <v>230.769</v>
       </c>
-      <c r="D19" s="5" t="n">
+      <c r="D19" s="27" t="n">
         <v>7891.85</v>
       </c>
-      <c r="E19" s="5" t="n">
+      <c r="E19" s="27" t="n">
         <v>12738.5</v>
       </c>
-      <c r="F19" t="n">
+      <c r="F19" s="26" t="n">
         <v>61.99987269792923</v>
       </c>
-      <c r="G19" s="8" t="n">
+      <c r="G19" s="28" t="n">
         <v>0.209586</v>
       </c>
-      <c r="H19" s="8" t="n">
+      <c r="H19" s="28" t="n">
         <v>0.7415119999999999</v>
       </c>
-      <c r="I19" s="8" t="n">
+      <c r="I19" s="28" t="n">
         <v>0.0489029</v>
       </c>
-      <c r="J19" s="8" t="n">
+      <c r="J19" s="28" t="n">
         <v>0.111603</v>
       </c>
-      <c r="K19" s="8" t="n">
+      <c r="K19" s="28" t="n">
         <v>0.7876570000000001</v>
       </c>
-      <c r="L19" s="8" t="n">
+      <c r="L19" s="28" t="n">
         <v>0.10074</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" t="n">
+      <c r="A20" s="13" t="n">
         <v>19</v>
       </c>
-      <c r="B20" s="5" t="n">
+      <c r="B20" s="23" t="n">
         <v>213.026</v>
       </c>
-      <c r="C20" s="5" t="n">
+      <c r="C20" s="23" t="n">
         <v>231.415</v>
       </c>
-      <c r="D20" s="5" t="n">
+      <c r="D20" s="23" t="n">
         <v>7976.47</v>
       </c>
-      <c r="E20" s="5" t="n">
+      <c r="E20" s="23" t="n">
         <v>12776.5</v>
       </c>
-      <c r="F20" t="n">
+      <c r="F20" s="13" t="n">
         <v>60.32437218809347</v>
       </c>
-      <c r="G20" s="8" t="n">
+      <c r="G20" s="25" t="n">
         <v>0.149831</v>
       </c>
-      <c r="H20" s="8" t="n">
+      <c r="H20" s="25" t="n">
         <v>0.788786</v>
       </c>
-      <c r="I20" s="8" t="n">
+      <c r="I20" s="25" t="n">
         <v>0.0613832</v>
       </c>
-      <c r="J20" s="8" t="n">
+      <c r="J20" s="25" t="n">
         <v>0.07752249999999999</v>
       </c>
-      <c r="K20" s="8" t="n">
+      <c r="K20" s="25" t="n">
         <v>0.802928</v>
       </c>
-      <c r="L20" s="8" t="n">
+      <c r="L20" s="25" t="n">
         <v>0.119549</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" t="n">
+      <c r="A21" s="26" t="n">
         <v>20</v>
       </c>
-      <c r="B21" s="5" t="n">
+      <c r="B21" s="27" t="n">
         <v>220.658</v>
       </c>
-      <c r="C21" s="5" t="n">
+      <c r="C21" s="27" t="n">
         <v>232.06</v>
       </c>
-      <c r="D21" s="5" t="n">
+      <c r="D21" s="27" t="n">
         <v>8014.56</v>
       </c>
-      <c r="E21" s="3" t="n">
+      <c r="E21" s="29" t="n">
         <v>0</v>
       </c>
-      <c r="F21" t="n">
+      <c r="F21" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="G21" s="8" t="n">
+      <c r="G21" s="28" t="n">
         <v>0.0953196</v>
       </c>
-      <c r="H21" s="8" t="n">
+      <c r="H21" s="28" t="n">
         <v>0.813125</v>
       </c>
-      <c r="I21" s="8" t="n">
+      <c r="I21" s="28" t="n">
         <v>0.0915552</v>
       </c>
-      <c r="J21" s="8" t="n">
+      <c r="J21" s="28" t="n">
         <v>0.0475694</v>
       </c>
-      <c r="K21" s="8" t="n">
+      <c r="K21" s="28" t="n">
         <v>0.785767</v>
       </c>
-      <c r="L21" s="8" t="n">
+      <c r="L21" s="28" t="n">
         <v>0.166664</v>
       </c>
     </row>
@@ -2218,172 +2722,173 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
+    <tabColor rgb="005B9BD5"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="9.28515625" defaultRowHeight="15"/>
   <cols>
-    <col width="30" bestFit="1" customWidth="1" min="1" max="1"/>
+    <col width="28" bestFit="1" customWidth="1" min="1" max="1"/>
     <col width="10" bestFit="1" customWidth="1" min="2" max="2"/>
-    <col width="11.5703125" bestFit="1" customWidth="1" min="3" max="3"/>
+    <col width="12" bestFit="1" customWidth="1" min="3" max="3"/>
     <col width="10" bestFit="1" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve"> Stream                     </t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">Feed </t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="30" t="inlineStr">
         <is>
           <t>Distillate</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">Bottom </t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+      <c r="A3" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve"> Stage                      </t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="B3" s="26" t="n">
         <v>12</v>
       </c>
-      <c r="C3" t="n">
+      <c r="C3" s="26" t="n">
         <v>1</v>
       </c>
-      <c r="D3" t="n">
+      <c r="D3" s="26" t="n">
         <v>20</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+      <c r="A4" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve"> Pressure (psia)            </t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="B4" s="13" t="n">
         <v>232.06</v>
       </c>
-      <c r="C4" t="n">
+      <c r="C4" s="13" t="n">
         <v>220.44</v>
       </c>
-      <c r="D4" t="n">
+      <c r="D4" s="13" t="n">
         <v>232.06</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+      <c r="A5" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve"> Vapour fraction        </t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="B5" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="C5" t="n">
+      <c r="C5" s="26" t="n">
         <v>0</v>
       </c>
-      <c r="D5" t="n">
+      <c r="D5" s="26" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="inlineStr">
+      <c r="A6" s="32" t="inlineStr">
         <is>
           <t xml:space="preserve"> Temperature (F)            </t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="B6" s="13" t="n">
         <v>174.999</v>
       </c>
-      <c r="C6" t="n">
+      <c r="C6" s="13" t="n">
         <v>118.74</v>
       </c>
-      <c r="D6" t="n">
+      <c r="D6" s="13" t="n">
         <v>220.653</v>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
+      <c r="A7" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve"> Total molar flow (lbmol/h) </t>
         </is>
       </c>
-      <c r="B7" t="n">
+      <c r="B7" s="26" t="n">
         <v>7142.98</v>
       </c>
-      <c r="C7" t="n">
+      <c r="C7" s="26" t="n">
         <v>2380.99</v>
       </c>
-      <c r="D7" t="n">
+      <c r="D7" s="26" t="n">
         <v>4761.98</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A9" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve"> Mole flows (lbmol/h)       </t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
+      <c r="A10" s="32" t="inlineStr">
         <is>
           <t>n-Propane</t>
         </is>
       </c>
-      <c r="B10" t="n">
+      <c r="B10" s="13" t="n">
         <v>2380.99</v>
       </c>
-      <c r="C10" s="9" t="n">
+      <c r="C10" s="33" t="n">
         <v>2154.47</v>
       </c>
-      <c r="D10" s="9" t="n">
+      <c r="D10" s="33" t="n">
         <v>226.525</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="inlineStr">
+      <c r="A11" s="31" t="inlineStr">
         <is>
           <t>n-Butane</t>
         </is>
       </c>
-      <c r="B11" t="n">
+      <c r="B11" s="26" t="n">
         <v>3968.32</v>
       </c>
-      <c r="C11" s="9" t="n">
+      <c r="C11" s="34" t="n">
         <v>226.511</v>
       </c>
-      <c r="D11" s="9" t="n">
+      <c r="D11" s="34" t="n">
         <v>3741.81</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr">
+      <c r="A12" s="32" t="inlineStr">
         <is>
           <t>N-Pentane</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B12" s="13" t="n">
         <v>793.664</v>
       </c>
-      <c r="C12" s="9" t="n">
+      <c r="C12" s="33" t="n">
         <v>0.0140691</v>
       </c>
-      <c r="D12" s="9" t="n">
+      <c r="D12" s="33" t="n">
         <v>793.65</v>
       </c>
     </row>

</xml_diff>